<commit_message>
feat: export published intent catalogs to Excel
</commit_message>
<xml_diff>
--- a/outputs/intent-catalog-template-20261025/tenant-intent-catalog-template.xlsx
+++ b/outputs/intent-catalog-template-20261025/tenant-intent-catalog-template.xlsx
@@ -2,18 +2,20 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2130184cdcfc4465"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intents" sheetId="2" r:id="Re0ab639a92074585"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="3" r:id="R2eed9fd65cca43ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="4" r:id="R17fcdf30ad204dfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relations" sheetId="5" r:id="R6a9ad312d8a2445e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkflowBindings" sheetId="6" r:id="R21a22ee8ddf44803"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QualityRules" sheetId="7" r:id="R8ab732d047d54bad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DocumentRequirements" sheetId="8" r:id="R15e7017457ec4739"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRMFieldMappings" sheetId="9" r:id="Re9dfdce5c8024fe0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChannelCapabilities" sheetId="10" r:id="R24e9e8f9b8cd4712"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestUtterances" sheetId="11" r:id="R9ed6dd1242dc4e9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CatalogManifest" sheetId="12" r:id="R58a007345ad14f88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R07bb3140e82742e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intents" sheetId="2" r:id="Ree9dc20a55e74c3e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Signals" sheetId="3" r:id="Rc0a7bacb3da54618"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Slots" sheetId="4" r:id="Rb0ebfbabcb7e4aba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relations" sheetId="5" r:id="Re9eae28a07ad44dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WorkflowBindings" sheetId="6" r:id="Ra8662163a9cf459b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QualityRules" sheetId="7" r:id="Rfed6fc5fc74e4f3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DocumentPolicies" sheetId="8" r:id="R75e74c63c7414cd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DocumentSettings" sheetId="9" r:id="Reed8c41299544ccc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DocumentRequirements" sheetId="10" r:id="R4a6f507acf6242bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CRMFieldMappings" sheetId="11" r:id="Rd7224f02784e4982"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChannelCapabilities" sheetId="12" r:id="Recfcc2814be34ed6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TestUtterances" sheetId="13" r:id="R80d28bae0b274c67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CatalogManifest" sheetId="14" r:id="R20dcc93632a24eb6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -362,7 +364,44 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="ChannelCapabilitiesTable" displayName="ChannelCapabilitiesTable" ref="A1:F5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="DocumentRequirementsTable" displayName="DocumentRequirementsTable" ref="A1:M5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:M5"/>
+  <x:tableColumns count="13">
+    <x:tableColumn id="1" name="intent_key"/>
+    <x:tableColumn id="2" name="requirement_key"/>
+    <x:tableColumn id="3" name="requirement_type"/>
+    <x:tableColumn id="4" name="required"/>
+    <x:tableColumn id="5" name="collection_order"/>
+    <x:tableColumn id="6" name="prompt_key"/>
+    <x:tableColumn id="7" name="validation_rule"/>
+    <x:tableColumn id="8" name="document_type"/>
+    <x:tableColumn id="9" name="fulfillment_mode"/>
+    <x:tableColumn id="10" name="next_intent_policy"/>
+    <x:tableColumn id="11" name="next_intent_keys"/>
+    <x:tableColumn id="12" name="source_of_truth"/>
+    <x:tableColumn id="13" name="notes"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="CRMFieldMappingsTable" displayName="CRMFieldMappingsTable" ref="A1:F7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F7"/>
+  <x:tableColumns count="6">
+    <x:tableColumn id="1" name="provider"/>
+    <x:tableColumn id="2" name="object_name"/>
+    <x:tableColumn id="3" name="source_field"/>
+    <x:tableColumn id="4" name="remote_field"/>
+    <x:tableColumn id="5" name="retention_class"/>
+    <x:tableColumn id="6" name="required"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="ChannelCapabilitiesTable" displayName="ChannelCapabilitiesTable" ref="A1:F5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:F5"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="channel"/>
@@ -376,8 +415,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="11" name="TestUtterancesTable" displayName="TestUtterancesTable" ref="A1:G10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="TestUtterancesTable" displayName="TestUtterancesTable" ref="A1:G10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:G10"/>
   <x:tableColumns count="7">
     <x:tableColumn id="1" name="test_id"/>
@@ -392,8 +431,8 @@
 </x:table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="CatalogManifestTable" displayName="CatalogManifestTable" ref="A1:B11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<file path=xl/tables/table14.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="14" name="CatalogManifestTable" displayName="CatalogManifestTable" ref="A1:B11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:autoFilter ref="A1:B11"/>
   <x:tableColumns count="2">
     <x:tableColumn id="1" name="key"/>
@@ -509,37 +548,50 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="DocumentRequirementsTable" displayName="DocumentRequirementsTable" ref="A1:M5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:M5"/>
-  <x:tableColumns count="13">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="DocumentPoliciesTable" displayName="DocumentPoliciesTable" ref="A1:O2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:O2"/>
+  <x:tableColumns count="15">
     <x:tableColumn id="1" name="intent_key"/>
-    <x:tableColumn id="2" name="requirement_key"/>
-    <x:tableColumn id="3" name="requirement_type"/>
-    <x:tableColumn id="4" name="required"/>
-    <x:tableColumn id="5" name="collection_order"/>
-    <x:tableColumn id="6" name="prompt_key"/>
-    <x:tableColumn id="7" name="validation_rule"/>
-    <x:tableColumn id="8" name="document_type"/>
-    <x:tableColumn id="9" name="fulfillment_mode"/>
-    <x:tableColumn id="10" name="next_intent_policy"/>
-    <x:tableColumn id="11" name="next_intent_keys"/>
-    <x:tableColumn id="12" name="source_of_truth"/>
-    <x:tableColumn id="13" name="notes"/>
+    <x:tableColumn id="2" name="enabled"/>
+    <x:tableColumn id="3" name="workflow_key"/>
+    <x:tableColumn id="4" name="request_mode"/>
+    <x:tableColumn id="5" name="required"/>
+    <x:tableColumn id="6" name="request_prompt_key"/>
+    <x:tableColumn id="7" name="allowed_document_types"/>
+    <x:tableColumn id="8" name="allow_user_initiated"/>
+    <x:tableColumn id="9" name="consent_required"/>
+    <x:tableColumn id="10" name="preserve_primary_intent"/>
+    <x:tableColumn id="11" name="store_extracted_text"/>
+    <x:tableColumn id="12" name="summary_target"/>
+    <x:tableColumn id="13" name="auto_create_lead"/>
+    <x:tableColumn id="14" name="auto_index_in_rag"/>
+    <x:tableColumn id="15" name="notes"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="CRMFieldMappingsTable" displayName="CRMFieldMappingsTable" ref="A1:F7" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:F7"/>
-  <x:tableColumns count="6">
-    <x:tableColumn id="1" name="provider"/>
-    <x:tableColumn id="2" name="object_name"/>
-    <x:tableColumn id="3" name="source_field"/>
-    <x:tableColumn id="4" name="remote_field"/>
-    <x:tableColumn id="5" name="retention_class"/>
-    <x:tableColumn id="6" name="required"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="DocumentSettingsTable" displayName="DocumentSettingsTable" ref="A1:Q2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:Q2"/>
+  <x:tableColumns count="17">
+    <x:tableColumn id="1" name="schema_version"/>
+    <x:tableColumn id="2" name="enabled"/>
+    <x:tableColumn id="3" name="storage_backend"/>
+    <x:tableColumn id="4" name="processing_provider"/>
+    <x:tableColumn id="5" name="workflow_key"/>
+    <x:tableColumn id="6" name="require_upload_consent"/>
+    <x:tableColumn id="7" name="max_file_bytes"/>
+    <x:tableColumn id="8" name="max_files_per_request"/>
+    <x:tableColumn id="9" name="max_pdf_pages"/>
+    <x:tableColumn id="10" name="ocr_languages"/>
+    <x:tableColumn id="11" name="allowed_mime_types"/>
+    <x:tableColumn id="12" name="retention_policy"/>
+    <x:tableColumn id="13" name="allow_public_document_urls"/>
+    <x:tableColumn id="14" name="allow_automatic_knowledge_ingestion"/>
+    <x:tableColumn id="15" name="allow_personal_identity_documents_by_default"/>
+    <x:tableColumn id="16" name="summary_rendering"/>
+    <x:tableColumn id="17" name="notes"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -787,7 +839,7 @@
         <x:v>Optional sheets</x:v>
       </x:c>
       <x:c r="B6" s="23" t="str">
-        <x:v>QualityRules, DocumentRequirements, CRMFieldMappings, ChannelCapabilities, TestUtterances, CatalogManifest</x:v>
+        <x:v>QualityRules, DocumentPolicies, DocumentSettings, DocumentRequirements, CRMFieldMappings, ChannelCapabilities, TestUtterances, CatalogManifest</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -841,12 +893,400 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4eca9427875f49da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab47ee5e308244e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="32" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="80" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A1" s="8" t="str">
+        <x:v>intent_key</x:v>
+      </x:c>
+      <x:c r="B1" s="29" t="str">
+        <x:v>requirement_key</x:v>
+      </x:c>
+      <x:c r="C1" s="29" t="str">
+        <x:v>requirement_type</x:v>
+      </x:c>
+      <x:c r="D1" s="29" t="str">
+        <x:v>required</x:v>
+      </x:c>
+      <x:c r="E1" s="29" t="str">
+        <x:v>collection_order</x:v>
+      </x:c>
+      <x:c r="F1" s="29" t="str">
+        <x:v>prompt_key</x:v>
+      </x:c>
+      <x:c r="G1" s="29" t="str">
+        <x:v>validation_rule</x:v>
+      </x:c>
+      <x:c r="H1" s="29" t="str">
+        <x:v>document_type</x:v>
+      </x:c>
+      <x:c r="I1" s="29" t="str">
+        <x:v>fulfillment_mode</x:v>
+      </x:c>
+      <x:c r="J1" s="29" t="str">
+        <x:v>next_intent_policy</x:v>
+      </x:c>
+      <x:c r="K1" s="29" t="str">
+        <x:v>next_intent_keys</x:v>
+      </x:c>
+      <x:c r="L1" s="29" t="str">
+        <x:v>source_of_truth</x:v>
+      </x:c>
+      <x:c r="M1" s="9" t="str">
+        <x:v>notes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="16" t="str">
+        <x:v>company.setup</x:v>
+      </x:c>
+      <x:c r="B2" s="33" t="str">
+        <x:v>company.documents.passport</x:v>
+      </x:c>
+      <x:c r="C2" s="33" t="str">
+        <x:v>document</x:v>
+      </x:c>
+      <x:c r="D2" s="34" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E2" s="33" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F2" s="33" t="str">
+        <x:v>document.ask_passport</x:v>
+      </x:c>
+      <x:c r="G2" s="33" t="str">
+        <x:v>document_type:passport</x:v>
+      </x:c>
+      <x:c r="H2" s="33" t="str">
+        <x:v>passport</x:v>
+      </x:c>
+      <x:c r="I2" s="33" t="str">
+        <x:v>external_confirmation_required</x:v>
+      </x:c>
+      <x:c r="J2" s="33" t="str">
+        <x:v>offer</x:v>
+      </x:c>
+      <x:c r="K2" s="33" t="str">
+        <x:v>document.intake</x:v>
+      </x:c>
+      <x:c r="L2" s="33" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="M2" s="17" t="str">
+        <x:v>Planning-template row. Runtime journey validation must be implemented before activation.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="16" t="str">
+        <x:v>company.setup</x:v>
+      </x:c>
+      <x:c r="B3" s="33" t="str">
+        <x:v>company.documents.identity</x:v>
+      </x:c>
+      <x:c r="C3" s="33" t="str">
+        <x:v>document</x:v>
+      </x:c>
+      <x:c r="D3" s="34" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E3" s="33" t="n">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="F3" s="33" t="str">
+        <x:v>document.ask_identity</x:v>
+      </x:c>
+      <x:c r="G3" s="33" t="str">
+        <x:v>document_type:identity</x:v>
+      </x:c>
+      <x:c r="H3" s="33" t="str">
+        <x:v>emirates_id_or_identity</x:v>
+      </x:c>
+      <x:c r="I3" s="33" t="str">
+        <x:v>external_confirmation_required</x:v>
+      </x:c>
+      <x:c r="J3" s="33" t="str">
+        <x:v>offer</x:v>
+      </x:c>
+      <x:c r="K3" s="33" t="str">
+        <x:v>document.intake</x:v>
+      </x:c>
+      <x:c r="L3" s="33" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="M3" s="17" t="str">
+        <x:v>Use only when the tenant policy requires it.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="16" t="str">
+        <x:v>company.setup</x:v>
+      </x:c>
+      <x:c r="B4" s="33" t="str">
+        <x:v>company.documents.ownership</x:v>
+      </x:c>
+      <x:c r="C4" s="33" t="str">
+        <x:v>document</x:v>
+      </x:c>
+      <x:c r="D4" s="34" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E4" s="33" t="n">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="F4" s="33" t="str">
+        <x:v>document.ask_ownership</x:v>
+      </x:c>
+      <x:c r="G4" s="33" t="str">
+        <x:v>document_type:ownership_declaration</x:v>
+      </x:c>
+      <x:c r="H4" s="33" t="str">
+        <x:v>ownership_declaration</x:v>
+      </x:c>
+      <x:c r="I4" s="33" t="str">
+        <x:v>external_confirmation_required</x:v>
+      </x:c>
+      <x:c r="J4" s="33" t="str">
+        <x:v>offer</x:v>
+      </x:c>
+      <x:c r="K4" s="33" t="str">
+        <x:v>document.intake</x:v>
+      </x:c>
+      <x:c r="L4" s="33" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="M4" s="17" t="str">
+        <x:v>Example ownership requirement.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="18" t="str">
+        <x:v>document.intake</x:v>
+      </x:c>
+      <x:c r="B5" s="35" t="str">
+        <x:v>document.upload.consent</x:v>
+      </x:c>
+      <x:c r="C5" s="35" t="str">
+        <x:v>consent</x:v>
+      </x:c>
+      <x:c r="D5" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E5" s="35" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F5" s="35" t="str">
+        <x:v>document.ask_consent</x:v>
+      </x:c>
+      <x:c r="G5" s="35" t="str">
+        <x:v>boolean:explicit_opt_in</x:v>
+      </x:c>
+      <x:c r="H5" s="35"/>
+      <x:c r="I5" s="35" t="str">
+        <x:v>conversation_ready</x:v>
+      </x:c>
+      <x:c r="J5" s="35" t="str">
+        <x:v>offer</x:v>
+      </x:c>
+      <x:c r="K5" s="35"/>
+      <x:c r="L5" s="35" t="str">
+        <x:v>tenant_catalog</x:v>
+      </x:c>
+      <x:c r="M5" s="19" t="str">
+        <x:v>Consent must be explicit and purpose-scoped.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7edccf27b51840d3"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="24" hidden="0" customHeight="1">
+      <x:c r="A1" s="8" t="str">
+        <x:v>provider</x:v>
+      </x:c>
+      <x:c r="B1" s="29" t="str">
+        <x:v>object_name</x:v>
+      </x:c>
+      <x:c r="C1" s="29" t="str">
+        <x:v>source_field</x:v>
+      </x:c>
+      <x:c r="D1" s="29" t="str">
+        <x:v>remote_field</x:v>
+      </x:c>
+      <x:c r="E1" s="29" t="str">
+        <x:v>retention_class</x:v>
+      </x:c>
+      <x:c r="F1" s="9" t="str">
+        <x:v>required</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="16" t="str">
+        <x:v>salesforce</x:v>
+      </x:c>
+      <x:c r="B2" s="33" t="str">
+        <x:v>Lead</x:v>
+      </x:c>
+      <x:c r="C2" s="33" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="D2" s="33" t="str">
+        <x:v>Name</x:v>
+      </x:c>
+      <x:c r="E2" s="33" t="str">
+        <x:v>pii</x:v>
+      </x:c>
+      <x:c r="F2" s="39" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="16" t="str">
+        <x:v>salesforce</x:v>
+      </x:c>
+      <x:c r="B3" s="33" t="str">
+        <x:v>Lead</x:v>
+      </x:c>
+      <x:c r="C3" s="33" t="str">
+        <x:v>email</x:v>
+      </x:c>
+      <x:c r="D3" s="33" t="str">
+        <x:v>Email</x:v>
+      </x:c>
+      <x:c r="E3" s="33" t="str">
+        <x:v>pii</x:v>
+      </x:c>
+      <x:c r="F3" s="39" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="16" t="str">
+        <x:v>salesforce</x:v>
+      </x:c>
+      <x:c r="B4" s="33" t="str">
+        <x:v>Lead</x:v>
+      </x:c>
+      <x:c r="C4" s="33" t="str">
+        <x:v>phone</x:v>
+      </x:c>
+      <x:c r="D4" s="33" t="str">
+        <x:v>Phone</x:v>
+      </x:c>
+      <x:c r="E4" s="33" t="str">
+        <x:v>pii</x:v>
+      </x:c>
+      <x:c r="F4" s="39" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="16" t="str">
+        <x:v>salesforce</x:v>
+      </x:c>
+      <x:c r="B5" s="33" t="str">
+        <x:v>Lead</x:v>
+      </x:c>
+      <x:c r="C5" s="33" t="str">
+        <x:v>interest_summary</x:v>
+      </x:c>
+      <x:c r="D5" s="33" t="str">
+        <x:v>Description</x:v>
+      </x:c>
+      <x:c r="E5" s="33" t="str">
+        <x:v>business</x:v>
+      </x:c>
+      <x:c r="F5" s="39" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="16" t="str">
+        <x:v>oracle</x:v>
+      </x:c>
+      <x:c r="B6" s="33" t="str">
+        <x:v>Lead</x:v>
+      </x:c>
+      <x:c r="C6" s="33" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="D6" s="33" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="E6" s="33" t="str">
+        <x:v>pii</x:v>
+      </x:c>
+      <x:c r="F6" s="39" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="18" t="str">
+        <x:v>sap</x:v>
+      </x:c>
+      <x:c r="B7" s="35" t="str">
+        <x:v>BusinessPartner</x:v>
+      </x:c>
+      <x:c r="C7" s="35" t="str">
+        <x:v>name</x:v>
+      </x:c>
+      <x:c r="D7" s="35" t="str">
+        <x:v>displayName</x:v>
+      </x:c>
+      <x:c r="E7" s="35" t="str">
+        <x:v>pii</x:v>
+      </x:c>
+      <x:c r="F7" s="40" t="b">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2af93d40a4c74241"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -961,12 +1401,12 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0bab546cae1a450f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R83271c94167e4325"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1206,12 +1646,12 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d6339ea25724dc7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9b9aa59cf4944e71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -1310,7 +1750,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7557fc06a2f44810"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4ae0fe5ada64ed5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1518,7 +1958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re95e64385d1a4cb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8beb6b3f3fff4a1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1947,7 +2387,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb19504d29dd648f7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7acf40ad66a646f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2518,7 +2958,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R182dd5f552d844fa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcf15d0de759a41ae"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2631,7 +3071,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb9c75aab446e4bd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18c6daac342f4892"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2756,7 +3196,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ea3bd280ee64a99"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1563c9b9649249a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2856,7 +3296,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R99f13cc8f1c34599"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7460e53b9df7426c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2866,225 +3306,120 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="34" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="20" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="34" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="32" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="22" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="20" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="80" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="22" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="20" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="26" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="20" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="80" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="24" hidden="0" customHeight="1">
+    <x:row r="1" ht="36" hidden="0" customHeight="1">
       <x:c r="A1" s="8" t="str">
         <x:v>intent_key</x:v>
       </x:c>
       <x:c r="B1" s="29" t="str">
-        <x:v>requirement_key</x:v>
+        <x:v>enabled</x:v>
       </x:c>
       <x:c r="C1" s="29" t="str">
-        <x:v>requirement_type</x:v>
+        <x:v>workflow_key</x:v>
       </x:c>
       <x:c r="D1" s="29" t="str">
+        <x:v>request_mode</x:v>
+      </x:c>
+      <x:c r="E1" s="29" t="str">
         <x:v>required</x:v>
       </x:c>
-      <x:c r="E1" s="29" t="str">
-        <x:v>collection_order</x:v>
-      </x:c>
       <x:c r="F1" s="29" t="str">
-        <x:v>prompt_key</x:v>
+        <x:v>request_prompt_key</x:v>
       </x:c>
       <x:c r="G1" s="29" t="str">
-        <x:v>validation_rule</x:v>
+        <x:v>allowed_document_types</x:v>
       </x:c>
       <x:c r="H1" s="29" t="str">
-        <x:v>document_type</x:v>
+        <x:v>allow_user_initiated</x:v>
       </x:c>
       <x:c r="I1" s="29" t="str">
-        <x:v>fulfillment_mode</x:v>
+        <x:v>consent_required</x:v>
       </x:c>
       <x:c r="J1" s="29" t="str">
-        <x:v>next_intent_policy</x:v>
+        <x:v>preserve_primary_intent</x:v>
       </x:c>
       <x:c r="K1" s="29" t="str">
-        <x:v>next_intent_keys</x:v>
+        <x:v>store_extracted_text</x:v>
       </x:c>
       <x:c r="L1" s="29" t="str">
-        <x:v>source_of_truth</x:v>
-      </x:c>
-      <x:c r="M1" s="9" t="str">
+        <x:v>summary_target</x:v>
+      </x:c>
+      <x:c r="M1" s="29" t="str">
+        <x:v>auto_create_lead</x:v>
+      </x:c>
+      <x:c r="N1" s="29" t="str">
+        <x:v>auto_index_in_rag</x:v>
+      </x:c>
+      <x:c r="O1" s="9" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="16" t="str">
+      <x:c r="A2" s="18" t="str">
         <x:v>company.setup</x:v>
       </x:c>
-      <x:c r="B2" s="33" t="str">
-        <x:v>company.documents.passport</x:v>
-      </x:c>
-      <x:c r="C2" s="33" t="str">
-        <x:v>document</x:v>
-      </x:c>
-      <x:c r="D2" s="34" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E2" s="33" t="n">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F2" s="33" t="str">
+      <x:c r="B2" s="36" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C2" s="35" t="str">
+        <x:v>document.intake</x:v>
+      </x:c>
+      <x:c r="D2" s="35" t="str">
+        <x:v>conditional_offer</x:v>
+      </x:c>
+      <x:c r="E2" s="36" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F2" s="35" t="str">
         <x:v>document.ask_passport</x:v>
       </x:c>
-      <x:c r="G2" s="33" t="str">
-        <x:v>document_type:passport</x:v>
-      </x:c>
-      <x:c r="H2" s="33" t="str">
-        <x:v>passport</x:v>
-      </x:c>
-      <x:c r="I2" s="33" t="str">
-        <x:v>external_confirmation_required</x:v>
-      </x:c>
-      <x:c r="J2" s="33" t="str">
-        <x:v>offer</x:v>
-      </x:c>
-      <x:c r="K2" s="33" t="str">
-        <x:v>document.intake</x:v>
-      </x:c>
-      <x:c r="L2" s="33" t="str">
-        <x:v>tenant_catalog</x:v>
-      </x:c>
-      <x:c r="M2" s="17" t="str">
-        <x:v>Planning-template row. Runtime journey validation must be implemented before activation.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="16" t="str">
-        <x:v>company.setup</x:v>
-      </x:c>
-      <x:c r="B3" s="33" t="str">
-        <x:v>company.documents.identity</x:v>
-      </x:c>
-      <x:c r="C3" s="33" t="str">
-        <x:v>document</x:v>
-      </x:c>
-      <x:c r="D3" s="34" t="b">
+      <x:c r="G2" s="35" t="str">
+        <x:v>["passport"]</x:v>
+      </x:c>
+      <x:c r="H2" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I2" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="J2" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="K2" s="36" t="b">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E3" s="33" t="n">
-        <x:v>21</x:v>
-      </x:c>
-      <x:c r="F3" s="33" t="str">
-        <x:v>document.ask_identity</x:v>
-      </x:c>
-      <x:c r="G3" s="33" t="str">
-        <x:v>document_type:identity</x:v>
-      </x:c>
-      <x:c r="H3" s="33" t="str">
-        <x:v>emirates_id_or_identity</x:v>
-      </x:c>
-      <x:c r="I3" s="33" t="str">
-        <x:v>external_confirmation_required</x:v>
-      </x:c>
-      <x:c r="J3" s="33" t="str">
-        <x:v>offer</x:v>
-      </x:c>
-      <x:c r="K3" s="33" t="str">
-        <x:v>document.intake</x:v>
-      </x:c>
-      <x:c r="L3" s="33" t="str">
-        <x:v>tenant_catalog</x:v>
-      </x:c>
-      <x:c r="M3" s="17" t="str">
-        <x:v>Use only when the tenant policy requires it.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="16" t="str">
-        <x:v>company.setup</x:v>
-      </x:c>
-      <x:c r="B4" s="33" t="str">
-        <x:v>company.documents.ownership</x:v>
-      </x:c>
-      <x:c r="C4" s="33" t="str">
-        <x:v>document</x:v>
-      </x:c>
-      <x:c r="D4" s="34" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E4" s="33" t="n">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="F4" s="33" t="str">
-        <x:v>document.ask_ownership</x:v>
-      </x:c>
-      <x:c r="G4" s="33" t="str">
-        <x:v>document_type:ownership_declaration</x:v>
-      </x:c>
-      <x:c r="H4" s="33" t="str">
-        <x:v>ownership_declaration</x:v>
-      </x:c>
-      <x:c r="I4" s="33" t="str">
-        <x:v>external_confirmation_required</x:v>
-      </x:c>
-      <x:c r="J4" s="33" t="str">
-        <x:v>offer</x:v>
-      </x:c>
-      <x:c r="K4" s="33" t="str">
-        <x:v>document.intake</x:v>
-      </x:c>
-      <x:c r="L4" s="33" t="str">
-        <x:v>tenant_catalog</x:v>
-      </x:c>
-      <x:c r="M4" s="17" t="str">
-        <x:v>Example ownership requirement.</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="18" t="str">
-        <x:v>document.intake</x:v>
-      </x:c>
-      <x:c r="B5" s="35" t="str">
-        <x:v>document.upload.consent</x:v>
-      </x:c>
-      <x:c r="C5" s="35" t="str">
-        <x:v>consent</x:v>
-      </x:c>
-      <x:c r="D5" s="36" t="b">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E5" s="35" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="F5" s="35" t="str">
-        <x:v>document.ask_consent</x:v>
-      </x:c>
-      <x:c r="G5" s="35" t="str">
-        <x:v>boolean:explicit_opt_in</x:v>
-      </x:c>
-      <x:c r="H5" s="35"/>
-      <x:c r="I5" s="35" t="str">
-        <x:v>conversation_ready</x:v>
-      </x:c>
-      <x:c r="J5" s="35" t="str">
-        <x:v>offer</x:v>
-      </x:c>
-      <x:c r="K5" s="35"/>
-      <x:c r="L5" s="35" t="str">
-        <x:v>tenant_catalog</x:v>
-      </x:c>
-      <x:c r="M5" s="19" t="str">
-        <x:v>Consent must be explicit and purpose-scoped.</x:v>
+      <x:c r="L2" s="35" t="str">
+        <x:v>crm_leads.summary</x:v>
+      </x:c>
+      <x:c r="M2" s="36" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="N2" s="36" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O2" s="19" t="str">
+        <x:v>Enable only after tenant document policy and OCR workflow review.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2e8c89e09acf4bfe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R89b9ab4abea84a10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3094,157 +3429,134 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="12" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="28" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="44" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="32" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="38" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="46" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="90" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="24" hidden="0" customHeight="1">
+    <x:row r="1" ht="60" hidden="0" customHeight="1">
       <x:c r="A1" s="8" t="str">
-        <x:v>provider</x:v>
+        <x:v>schema_version</x:v>
       </x:c>
       <x:c r="B1" s="29" t="str">
-        <x:v>object_name</x:v>
+        <x:v>enabled</x:v>
       </x:c>
       <x:c r="C1" s="29" t="str">
-        <x:v>source_field</x:v>
+        <x:v>storage_backend</x:v>
       </x:c>
       <x:c r="D1" s="29" t="str">
-        <x:v>remote_field</x:v>
+        <x:v>processing_provider</x:v>
       </x:c>
       <x:c r="E1" s="29" t="str">
-        <x:v>retention_class</x:v>
-      </x:c>
-      <x:c r="F1" s="9" t="str">
-        <x:v>required</x:v>
+        <x:v>workflow_key</x:v>
+      </x:c>
+      <x:c r="F1" s="29" t="str">
+        <x:v>require_upload_consent</x:v>
+      </x:c>
+      <x:c r="G1" s="29" t="str">
+        <x:v>max_file_bytes</x:v>
+      </x:c>
+      <x:c r="H1" s="29" t="str">
+        <x:v>max_files_per_request</x:v>
+      </x:c>
+      <x:c r="I1" s="29" t="str">
+        <x:v>max_pdf_pages</x:v>
+      </x:c>
+      <x:c r="J1" s="29" t="str">
+        <x:v>ocr_languages</x:v>
+      </x:c>
+      <x:c r="K1" s="29" t="str">
+        <x:v>allowed_mime_types</x:v>
+      </x:c>
+      <x:c r="L1" s="29" t="str">
+        <x:v>retention_policy</x:v>
+      </x:c>
+      <x:c r="M1" s="29" t="str">
+        <x:v>allow_public_document_urls</x:v>
+      </x:c>
+      <x:c r="N1" s="29" t="str">
+        <x:v>allow_automatic_knowledge_ingestion</x:v>
+      </x:c>
+      <x:c r="O1" s="29" t="str">
+        <x:v>allow_personal_identity_documents_by_default</x:v>
+      </x:c>
+      <x:c r="P1" s="29" t="str">
+        <x:v>summary_rendering</x:v>
+      </x:c>
+      <x:c r="Q1" s="9" t="str">
+        <x:v>notes</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
-      <x:c r="A2" s="16" t="str">
-        <x:v>salesforce</x:v>
-      </x:c>
-      <x:c r="B2" s="33" t="str">
-        <x:v>Lead</x:v>
-      </x:c>
-      <x:c r="C2" s="33" t="str">
-        <x:v>name</x:v>
-      </x:c>
-      <x:c r="D2" s="33" t="str">
-        <x:v>Name</x:v>
-      </x:c>
-      <x:c r="E2" s="33" t="str">
-        <x:v>pii</x:v>
-      </x:c>
-      <x:c r="F2" s="39" t="b">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="16" t="str">
-        <x:v>salesforce</x:v>
-      </x:c>
-      <x:c r="B3" s="33" t="str">
-        <x:v>Lead</x:v>
-      </x:c>
-      <x:c r="C3" s="33" t="str">
-        <x:v>email</x:v>
-      </x:c>
-      <x:c r="D3" s="33" t="str">
-        <x:v>Email</x:v>
-      </x:c>
-      <x:c r="E3" s="33" t="str">
-        <x:v>pii</x:v>
-      </x:c>
-      <x:c r="F3" s="39" t="b">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="16" t="str">
-        <x:v>salesforce</x:v>
-      </x:c>
-      <x:c r="B4" s="33" t="str">
-        <x:v>Lead</x:v>
-      </x:c>
-      <x:c r="C4" s="33" t="str">
-        <x:v>phone</x:v>
-      </x:c>
-      <x:c r="D4" s="33" t="str">
-        <x:v>Phone</x:v>
-      </x:c>
-      <x:c r="E4" s="33" t="str">
-        <x:v>pii</x:v>
-      </x:c>
-      <x:c r="F4" s="39" t="b">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="16" t="str">
-        <x:v>salesforce</x:v>
-      </x:c>
-      <x:c r="B5" s="33" t="str">
-        <x:v>Lead</x:v>
-      </x:c>
-      <x:c r="C5" s="33" t="str">
-        <x:v>interest_summary</x:v>
-      </x:c>
-      <x:c r="D5" s="33" t="str">
-        <x:v>Description</x:v>
-      </x:c>
-      <x:c r="E5" s="33" t="str">
-        <x:v>business</x:v>
-      </x:c>
-      <x:c r="F5" s="39" t="b">
+      <x:c r="A2" s="18" t="str">
+        <x:v>document-v1</x:v>
+      </x:c>
+      <x:c r="B2" s="36" t="b">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="16" t="str">
-        <x:v>oracle</x:v>
-      </x:c>
-      <x:c r="B6" s="33" t="str">
-        <x:v>Lead</x:v>
-      </x:c>
-      <x:c r="C6" s="33" t="str">
-        <x:v>name</x:v>
-      </x:c>
-      <x:c r="D6" s="33" t="str">
-        <x:v>name</x:v>
-      </x:c>
-      <x:c r="E6" s="33" t="str">
-        <x:v>pii</x:v>
-      </x:c>
-      <x:c r="F6" s="39" t="b">
+      <x:c r="C2" s="35" t="str">
+        <x:v>private_server_storage</x:v>
+      </x:c>
+      <x:c r="D2" s="35" t="str">
+        <x:v>python_tesseract</x:v>
+      </x:c>
+      <x:c r="E2" s="35" t="str">
+        <x:v>document.intake</x:v>
+      </x:c>
+      <x:c r="F2" s="36" t="b">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="G2" s="35" t="n">
+        <x:v>10000000</x:v>
+      </x:c>
+      <x:c r="H2" s="35" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I2" s="35" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J2" s="35" t="str">
+        <x:v>["eng"]</x:v>
+      </x:c>
+      <x:c r="K2" s="35" t="str">
+        <x:v>["application/pdf","image/jpeg","image/png"]</x:v>
+      </x:c>
+      <x:c r="L2" s="35" t="str">
+        <x:v>tenant_configured</x:v>
+      </x:c>
+      <x:c r="M2" s="36" t="b">
         <x:v>0</x:v>
       </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="18" t="str">
-        <x:v>sap</x:v>
-      </x:c>
-      <x:c r="B7" s="35" t="str">
-        <x:v>BusinessPartner</x:v>
-      </x:c>
-      <x:c r="C7" s="35" t="str">
-        <x:v>name</x:v>
-      </x:c>
-      <x:c r="D7" s="35" t="str">
-        <x:v>displayName</x:v>
-      </x:c>
-      <x:c r="E7" s="35" t="str">
-        <x:v>pii</x:v>
-      </x:c>
-      <x:c r="F7" s="40" t="b">
+      <x:c r="N2" s="36" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="O2" s="36" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="P2" s="35" t="str">
+        <x:v>conversation_plus_redacted_document_excerpts</x:v>
+      </x:c>
+      <x:c r="Q2" s="19" t="str">
+        <x:v>Enable only after storage, consent, OCR and retention review.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3eb68ff9ef934d0a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re56331ea4bec45d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>